<commit_message>
chore: update hour log
</commit_message>
<xml_diff>
--- a/DTT-Assessment-Hour-Log.xlsx
+++ b/DTT-Assessment-Hour-Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bae1ac55f5db4960/Desktop/DTT_assessment/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dtt-frontend-assessment\dtt-frontend-assessment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{49F91033-96F3-7148-A020-201798871A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF858867-1A1D-45F4-9E64-E6575D8DC05A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D68B41-DA8C-4C9E-9D96-22C4924DD0A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19125" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="28800" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DTT Test Hour Log" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Subject</t>
   </si>
@@ -111,6 +111,12 @@
   <si>
     <t>18/05/2026</t>
   </si>
+  <si>
+    <t>Assets setup</t>
+  </si>
+  <si>
+    <t>Added DTT provided icons and images to src/assets folder, organized into icons and images subfolders</t>
+  </si>
 </sst>
 </file>
 
@@ -118,7 +124,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -450,6 +456,12 @@
     <xf numFmtId="49" fontId="11" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -461,12 +473,6 @@
     </xf>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1737,22 +1743,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
+      <c r="A1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
       <c r="E1" s="10"/>
       <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:6" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="25"/>
     </row>
     <row r="3" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
@@ -1776,7 +1782,7 @@
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="25">
+      <c r="B4" s="21">
         <v>0.5</v>
       </c>
       <c r="C4" s="17" t="s">
@@ -1792,7 +1798,7 @@
       <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="21">
         <v>1</v>
       </c>
       <c r="C5" s="17" t="s">
@@ -1808,7 +1814,7 @@
       <c r="A6" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="21">
         <v>0.5</v>
       </c>
       <c r="C6" s="17" t="s">
@@ -1824,7 +1830,7 @@
       <c r="A7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="21">
         <v>0.5</v>
       </c>
       <c r="C7" s="17" t="s">
@@ -1840,7 +1846,7 @@
       <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="21">
         <v>0.5</v>
       </c>
       <c r="C8" s="17" t="s">
@@ -1853,24 +1859,32 @@
       <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="5"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="15"/>
+      <c r="A9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="21">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>20</v>
+      </c>
       <c r="E9" s="19"/>
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5"/>
-      <c r="B10" s="25"/>
+      <c r="B10" s="21"/>
       <c r="C10" s="17"/>
-      <c r="D10" s="24"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="19"/>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
-      <c r="B11" s="25"/>
+      <c r="B11" s="21"/>
       <c r="C11" s="17"/>
       <c r="D11" s="15"/>
       <c r="E11" s="19"/>
@@ -1878,7 +1892,7 @@
     </row>
     <row r="12" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
-      <c r="B12" s="25"/>
+      <c r="B12" s="21"/>
       <c r="C12" s="17"/>
       <c r="D12" s="15"/>
       <c r="E12" s="19"/>
@@ -1886,7 +1900,7 @@
     </row>
     <row r="13" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5"/>
-      <c r="B13" s="25"/>
+      <c r="B13" s="21"/>
       <c r="C13" s="17"/>
       <c r="D13" s="15"/>
       <c r="E13" s="19"/>
@@ -1894,7 +1908,7 @@
     </row>
     <row r="14" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
-      <c r="B14" s="25"/>
+      <c r="B14" s="21"/>
       <c r="C14" s="17"/>
       <c r="D14" s="15"/>
       <c r="E14" s="19"/>
@@ -1902,7 +1916,7 @@
     </row>
     <row r="15" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
-      <c r="B15" s="25"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="17"/>
       <c r="D15" s="15"/>
       <c r="E15" s="19"/>
@@ -1910,7 +1924,7 @@
     </row>
     <row r="16" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5"/>
-      <c r="B16" s="25"/>
+      <c r="B16" s="21"/>
       <c r="C16" s="17"/>
       <c r="D16" s="15"/>
       <c r="E16" s="19"/>
@@ -1918,7 +1932,7 @@
     </row>
     <row r="17" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
-      <c r="B17" s="25"/>
+      <c r="B17" s="21"/>
       <c r="C17" s="17"/>
       <c r="D17" s="15"/>
       <c r="E17" s="19"/>
@@ -1926,7 +1940,7 @@
     </row>
     <row r="18" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5"/>
-      <c r="B18" s="25"/>
+      <c r="B18" s="21"/>
       <c r="C18" s="17"/>
       <c r="D18" s="15"/>
       <c r="E18" s="19"/>
@@ -1934,7 +1948,7 @@
     </row>
     <row r="19" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5"/>
-      <c r="B19" s="25"/>
+      <c r="B19" s="21"/>
       <c r="C19" s="17"/>
       <c r="D19" s="15"/>
       <c r="E19" s="19"/>
@@ -1942,7 +1956,7 @@
     </row>
     <row r="20" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
-      <c r="B20" s="25"/>
+      <c r="B20" s="21"/>
       <c r="C20" s="17"/>
       <c r="D20" s="15"/>
       <c r="E20" s="19"/>
@@ -1950,7 +1964,7 @@
     </row>
     <row r="21" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5"/>
-      <c r="B21" s="25"/>
+      <c r="B21" s="21"/>
       <c r="C21" s="17"/>
       <c r="D21" s="15"/>
       <c r="E21" s="19"/>
@@ -1958,7 +1972,7 @@
     </row>
     <row r="22" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
-      <c r="B22" s="25"/>
+      <c r="B22" s="21"/>
       <c r="C22" s="17"/>
       <c r="D22" s="15"/>
       <c r="E22" s="19"/>
@@ -1966,7 +1980,7 @@
     </row>
     <row r="23" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
-      <c r="B23" s="25"/>
+      <c r="B23" s="21"/>
       <c r="C23" s="17"/>
       <c r="D23" s="15"/>
       <c r="E23" s="19"/>
@@ -1974,7 +1988,7 @@
     </row>
     <row r="24" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
-      <c r="B24" s="25"/>
+      <c r="B24" s="21"/>
       <c r="C24" s="17"/>
       <c r="D24" s="15"/>
       <c r="E24" s="19"/>
@@ -1982,7 +1996,7 @@
     </row>
     <row r="25" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
-      <c r="B25" s="25"/>
+      <c r="B25" s="21"/>
       <c r="C25" s="17"/>
       <c r="D25" s="15"/>
       <c r="E25" s="19"/>
@@ -1990,7 +2004,7 @@
     </row>
     <row r="26" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
-      <c r="B26" s="25"/>
+      <c r="B26" s="21"/>
       <c r="C26" s="17"/>
       <c r="D26" s="15"/>
       <c r="E26" s="19"/>
@@ -1998,7 +2012,7 @@
     </row>
     <row r="27" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
-      <c r="B27" s="25"/>
+      <c r="B27" s="21"/>
       <c r="C27" s="17"/>
       <c r="D27" s="15"/>
       <c r="E27" s="19"/>
@@ -2006,7 +2020,7 @@
     </row>
     <row r="28" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
-      <c r="B28" s="25"/>
+      <c r="B28" s="21"/>
       <c r="C28" s="17"/>
       <c r="D28" s="15"/>
       <c r="E28" s="19"/>
@@ -2026,7 +2040,7 @@
       </c>
       <c r="B30" s="14">
         <f>SUMIF(E4:E28,"&lt;&gt;x",B4:B28)</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>

</xml_diff>